<commit_message>
Add product weights to USP listing (Set 2 from Gautam's sheet)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KXQyatQdYSKeTsiHbQVdrE
</commit_message>
<xml_diff>
--- a/listing/USP/USP_Listings.xlsx
+++ b/listing/USP/USP_Listings.xlsx
@@ -588,7 +588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -598,8 +598,9 @@
     <col width="80" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -654,10 +655,15 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
+          <t>Weight (kg)</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
           <t>Images</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>Image folder</t>
         </is>
@@ -676,7 +682,8 @@
       <c r="F5" s="5" t="n"/>
       <c r="G5" s="5" t="n"/>
       <c r="H5" s="5" t="n"/>
-      <c r="I5" s="6" t="n"/>
+      <c r="I5" s="5" t="n"/>
+      <c r="J5" s="6" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
@@ -711,9 +718,12 @@
         </is>
       </c>
       <c r="H6" s="7" t="n">
+        <v>18</v>
+      </c>
+      <c r="I6" s="7" t="n">
         <v>14</v>
       </c>
-      <c r="I6" s="11" t="inlineStr">
+      <c r="J6" s="11" t="inlineStr">
         <is>
           <t>images/01_SS_GT_35L_GT53H3</t>
         </is>
@@ -751,10 +761,15 @@
           <t>Catalogue</t>
         </is>
       </c>
-      <c r="H7" s="7" t="n">
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="n">
         <v>14</v>
       </c>
-      <c r="I7" s="11" t="inlineStr">
+      <c r="J7" s="11" t="inlineStr">
         <is>
           <t>images/02_SS_GT_60L_GT743</t>
         </is>
@@ -792,10 +807,15 @@
           <t>Catalogue</t>
         </is>
       </c>
-      <c r="H8" s="7" t="n">
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="n">
         <v>14</v>
       </c>
-      <c r="I8" s="11" t="inlineStr">
+      <c r="J8" s="11" t="inlineStr">
         <is>
           <t>images/03_SS_GT_85L_GT84H3H</t>
         </is>
@@ -833,10 +853,15 @@
           <t>Catalogue</t>
         </is>
       </c>
-      <c r="H9" s="7" t="n">
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="I9" s="11" t="inlineStr">
+      <c r="J9" s="11" t="inlineStr">
         <is>
           <t>images/04_SS_DG_300_DG11</t>
         </is>
@@ -874,10 +899,15 @@
           <t>Catalogue</t>
         </is>
       </c>
-      <c r="H10" s="7" t="n">
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="I10" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="I10" s="11" t="inlineStr">
+      <c r="J10" s="11" t="inlineStr">
         <is>
           <t>images/05_SS_DG_600_DG21</t>
         </is>
@@ -917,10 +947,15 @@
           <t>To confirm (1050 mm size not in catalogue)</t>
         </is>
       </c>
-      <c r="H11" s="7" t="n">
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="I11" s="11" t="inlineStr">
+      <c r="J11" s="11" t="inlineStr">
         <is>
           <t>images/06_SS_WT_US2_1050</t>
         </is>
@@ -958,10 +993,15 @@
           <t>28 Oct 2026 update</t>
         </is>
       </c>
-      <c r="H12" s="7" t="n">
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="I12" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="I12" s="11" t="inlineStr">
+      <c r="J12" s="11" t="inlineStr">
         <is>
           <t>images/07_SS_5TR_900_5TR3</t>
         </is>
@@ -999,10 +1039,15 @@
           <t>28 Oct 2026 update</t>
         </is>
       </c>
-      <c r="H13" s="7" t="n">
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="I13" s="11" t="inlineStr">
+      <c r="J13" s="11" t="inlineStr">
         <is>
           <t>images/08_SS_5TR_1150_5TR4</t>
         </is>
@@ -1040,10 +1085,15 @@
           <t>28 Oct 2026 update</t>
         </is>
       </c>
-      <c r="H14" s="7" t="n">
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="I14" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="I14" s="11" t="inlineStr">
+      <c r="J14" s="11" t="inlineStr">
         <is>
           <t>images/09_MS_5TR_900_MSR94H</t>
         </is>
@@ -1081,10 +1131,15 @@
           <t>28 Oct 2026 update</t>
         </is>
       </c>
-      <c r="H15" s="7" t="n">
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="I15" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="I15" s="11" t="inlineStr">
+      <c r="J15" s="11" t="inlineStr">
         <is>
           <t>images/10_MS_5TR_1200_MSR124H</t>
         </is>
@@ -1103,7 +1158,8 @@
       <c r="F16" s="5" t="n"/>
       <c r="G16" s="5" t="n"/>
       <c r="H16" s="5" t="n"/>
-      <c r="I16" s="6" t="n"/>
+      <c r="I16" s="5" t="n"/>
+      <c r="J16" s="6" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="n">
@@ -1138,9 +1194,12 @@
         </is>
       </c>
       <c r="H17" s="7" t="n">
+        <v>29</v>
+      </c>
+      <c r="I17" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="I17" s="11" t="inlineStr">
+      <c r="J17" s="11" t="inlineStr">
         <is>
           <t>images/11_SS_WT_CS_OHS2_BS_900_3WTCO2B</t>
         </is>
@@ -1179,9 +1238,12 @@
         </is>
       </c>
       <c r="H18" s="7" t="n">
+        <v>34</v>
+      </c>
+      <c r="I18" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="I18" s="11" t="inlineStr">
+      <c r="J18" s="11" t="inlineStr">
         <is>
           <t>images/12_SS_WT_CS_OHS2_BS_1150_4WTCO2B</t>
         </is>
@@ -1220,9 +1282,12 @@
         </is>
       </c>
       <c r="H19" s="7" t="n">
+        <v>41</v>
+      </c>
+      <c r="I19" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="I19" s="11" t="inlineStr">
+      <c r="J19" s="11" t="inlineStr">
         <is>
           <t>images/13_SS_WT_CS_OHS2_BS_1500_5WTCO2B</t>
         </is>
@@ -1261,9 +1326,12 @@
         </is>
       </c>
       <c r="H20" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="I20" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="I20" s="11" t="inlineStr">
+      <c r="J20" s="11" t="inlineStr">
         <is>
           <t>images/14_SS_WT_US1_OHS2_BS_900_3WTU1O2B</t>
         </is>
@@ -1302,9 +1370,12 @@
         </is>
       </c>
       <c r="H21" s="7" t="n">
+        <v>37</v>
+      </c>
+      <c r="I21" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="I21" s="11" t="inlineStr">
+      <c r="J21" s="11" t="inlineStr">
         <is>
           <t>images/15_SS_WT_US1_OHS2_BS_1150_4WTU1O2B</t>
         </is>
@@ -1343,9 +1414,12 @@
         </is>
       </c>
       <c r="H22" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="I22" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="I22" s="11" t="inlineStr">
+      <c r="J22" s="11" t="inlineStr">
         <is>
           <t>images/16_SS_WT_US1_OHS2_BS_1500_5WTU1O2B</t>
         </is>
@@ -1384,9 +1458,12 @@
         </is>
       </c>
       <c r="H23" s="7" t="n">
+        <v>36</v>
+      </c>
+      <c r="I23" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="I23" s="11" t="inlineStr">
+      <c r="J23" s="11" t="inlineStr">
         <is>
           <t>images/17_SS_WT_US2_OHS2_BS_900_3WTU2O2B</t>
         </is>
@@ -1425,9 +1502,12 @@
         </is>
       </c>
       <c r="H24" s="7" t="n">
+        <v>43</v>
+      </c>
+      <c r="I24" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="I24" s="11" t="inlineStr">
+      <c r="J24" s="11" t="inlineStr">
         <is>
           <t>images/18_SS_WT_US2_OHS2_BS_1150_4WTU2O2B</t>
         </is>
@@ -1466,9 +1546,12 @@
         </is>
       </c>
       <c r="H25" s="7" t="n">
+        <v>53</v>
+      </c>
+      <c r="I25" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="I25" s="11" t="inlineStr">
+      <c r="J25" s="11" t="inlineStr">
         <is>
           <t>images/19_SS_WT_US2_OHS2_BS_1500_5WTU2O2B</t>
         </is>
@@ -1507,9 +1590,12 @@
         </is>
       </c>
       <c r="H26" s="7" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="I26" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="I26" s="11" t="inlineStr">
+      <c r="J26" s="11" t="inlineStr">
         <is>
           <t>images/20_SS_OHS2_900_3OHS2</t>
         </is>
@@ -1548,9 +1634,12 @@
         </is>
       </c>
       <c r="H27" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="I27" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="I27" s="11" t="inlineStr">
+      <c r="J27" s="11" t="inlineStr">
         <is>
           <t>images/21_SS_OHS2_1150_4OHS2</t>
         </is>
@@ -1589,9 +1678,12 @@
         </is>
       </c>
       <c r="H28" s="7" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="I28" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="I28" s="11" t="inlineStr">
+      <c r="J28" s="11" t="inlineStr">
         <is>
           <t>images/22_SS_OHS2_1500_5OHS2</t>
         </is>
@@ -1599,8 +1691,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A5:I5"/>
-    <mergeCell ref="A16:I16"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A16:J16"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId1"/>
@@ -2700,7 +2792,11 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="18" t="n"/>
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>29 kg</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="13">
@@ -3098,7 +3194,11 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="18" t="n"/>
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>34 kg</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="13">
@@ -3496,7 +3596,11 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="18" t="n"/>
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>41 kg</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="13">
@@ -3894,7 +3998,11 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="18" t="n"/>
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>30 kg</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="13">
@@ -4292,7 +4400,11 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="18" t="n"/>
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>37 kg</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="13">
@@ -4690,7 +4802,11 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="18" t="n"/>
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>45 kg</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="13">
@@ -5088,7 +5204,11 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="18" t="n"/>
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>36 kg</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="13">
@@ -5486,7 +5606,11 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="18" t="n"/>
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>43 kg</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="13">
@@ -5910,7 +6034,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>18 Kgs</t>
+          <t>18 kg</t>
         </is>
       </c>
     </row>
@@ -6310,7 +6434,11 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="18" t="n"/>
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>53 kg</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="13">
@@ -6692,7 +6820,11 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="18" t="n"/>
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>12.5 kg</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="11">
@@ -7072,7 +7204,11 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="18" t="n"/>
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>15 kg</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="11">
@@ -7452,7 +7588,11 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="18" t="n"/>
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>18.5 kg</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="11">

</xml_diff>

<commit_message>
Set 2 weights now include 5 kg packing material
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KXQyatQdYSKeTsiHbQVdrE
</commit_message>
<xml_diff>
--- a/listing/USP/USP_Listings.xlsx
+++ b/listing/USP/USP_Listings.xlsx
@@ -613,7 +613,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Prices in Rs, excl. GST (18% extra), shipping, unloading and installation. Image folders are in images/ under the same S.No.</t>
+          <t>Prices in Rs, excl. GST (18% extra), shipping, unloading and installation. Image folders are in images/ under the same S.No. Set 2 weights include 5 kg packing material; the Set 1 weight (GT53H3) is the product weight.</t>
         </is>
       </c>
     </row>
@@ -1194,7 +1194,7 @@
         </is>
       </c>
       <c r="H17" s="7" t="n">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="I17" s="7" t="n">
         <v>6</v>
@@ -1238,7 +1238,7 @@
         </is>
       </c>
       <c r="H18" s="7" t="n">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="I18" s="7" t="n">
         <v>6</v>
@@ -1282,7 +1282,7 @@
         </is>
       </c>
       <c r="H19" s="7" t="n">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="I19" s="7" t="n">
         <v>6</v>
@@ -1326,7 +1326,7 @@
         </is>
       </c>
       <c r="H20" s="7" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="I20" s="7" t="n">
         <v>7</v>
@@ -1370,7 +1370,7 @@
         </is>
       </c>
       <c r="H21" s="7" t="n">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="I21" s="7" t="n">
         <v>7</v>
@@ -1414,7 +1414,7 @@
         </is>
       </c>
       <c r="H22" s="7" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="I22" s="7" t="n">
         <v>7</v>
@@ -1458,7 +1458,7 @@
         </is>
       </c>
       <c r="H23" s="7" t="n">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="I23" s="7" t="n">
         <v>7</v>
@@ -1502,7 +1502,7 @@
         </is>
       </c>
       <c r="H24" s="7" t="n">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="I24" s="7" t="n">
         <v>7</v>
@@ -1546,7 +1546,7 @@
         </is>
       </c>
       <c r="H25" s="7" t="n">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="I25" s="7" t="n">
         <v>7</v>
@@ -1590,7 +1590,7 @@
         </is>
       </c>
       <c r="H26" s="7" t="n">
-        <v>12.5</v>
+        <v>17.5</v>
       </c>
       <c r="I26" s="7" t="n">
         <v>8</v>
@@ -1634,7 +1634,7 @@
         </is>
       </c>
       <c r="H27" s="7" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="I27" s="7" t="n">
         <v>8</v>
@@ -1678,7 +1678,7 @@
         </is>
       </c>
       <c r="H28" s="7" t="n">
-        <v>18.5</v>
+        <v>23.5</v>
       </c>
       <c r="I28" s="7" t="n">
         <v>8</v>
@@ -2794,7 +2794,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>29 kg</t>
+          <t>34 kg (incl. 5 kg packing; product 29 kg)</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>34 kg</t>
+          <t>39 kg (incl. 5 kg packing; product 34 kg)</t>
         </is>
       </c>
     </row>
@@ -3598,7 +3598,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>41 kg</t>
+          <t>46 kg (incl. 5 kg packing; product 41 kg)</t>
         </is>
       </c>
     </row>
@@ -4000,7 +4000,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>30 kg</t>
+          <t>35 kg (incl. 5 kg packing; product 30 kg)</t>
         </is>
       </c>
     </row>
@@ -4402,7 +4402,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>37 kg</t>
+          <t>42 kg (incl. 5 kg packing; product 37 kg)</t>
         </is>
       </c>
     </row>
@@ -4804,7 +4804,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>45 kg</t>
+          <t>50 kg (incl. 5 kg packing; product 45 kg)</t>
         </is>
       </c>
     </row>
@@ -5206,7 +5206,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>36 kg</t>
+          <t>41 kg (incl. 5 kg packing; product 36 kg)</t>
         </is>
       </c>
     </row>
@@ -5608,7 +5608,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>43 kg</t>
+          <t>48 kg (incl. 5 kg packing; product 43 kg)</t>
         </is>
       </c>
     </row>
@@ -6436,7 +6436,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>53 kg</t>
+          <t>58 kg (incl. 5 kg packing; product 53 kg)</t>
         </is>
       </c>
     </row>
@@ -6822,7 +6822,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>12.5 kg</t>
+          <t>17.5 kg (incl. 5 kg packing; product 12.5 kg)</t>
         </is>
       </c>
     </row>
@@ -7206,7 +7206,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>15 kg</t>
+          <t>20 kg (incl. 5 kg packing; product 15 kg)</t>
         </is>
       </c>
     </row>
@@ -7590,7 +7590,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>18.5 kg</t>
+          <t>23.5 kg (incl. 5 kg packing; product 18.5 kg)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Set 1 packed weights and coupling corrections from 22 Oct sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KXQyatQdYSKeTsiHbQVdrE
</commit_message>
<xml_diff>
--- a/listing/USP/USP_Listings.xlsx
+++ b/listing/USP/USP_Listings.xlsx
@@ -613,7 +613,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Prices in Rs, excl. GST (18% extra), shipping, unloading and installation. Image folders are in images/ under the same S.No. Set 2 weights include 5 kg packing material; the Set 1 weight (GT53H3) is the product weight.</t>
+          <t>Prices in Rs, excl. GST (18% extra), shipping, unloading and installation. Image folders are in images/ under the same S.No. All weights include packing material.</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Weight (kg)</t>
+          <t>Weight incl. packing (kg)</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
@@ -761,10 +761,8 @@
           <t>Catalogue</t>
         </is>
       </c>
-      <c r="H7" s="7" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
+      <c r="H7" s="7" t="n">
+        <v>23</v>
       </c>
       <c r="I7" s="7" t="n">
         <v>14</v>
@@ -807,10 +805,8 @@
           <t>Catalogue</t>
         </is>
       </c>
-      <c r="H8" s="7" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
+      <c r="H8" s="7" t="n">
+        <v>27</v>
       </c>
       <c r="I8" s="7" t="n">
         <v>14</v>
@@ -853,10 +849,8 @@
           <t>Catalogue</t>
         </is>
       </c>
-      <c r="H9" s="7" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
+      <c r="H9" s="7" t="n">
+        <v>7</v>
       </c>
       <c r="I9" s="7" t="n">
         <v>7</v>
@@ -899,10 +893,8 @@
           <t>Catalogue</t>
         </is>
       </c>
-      <c r="H10" s="7" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
+      <c r="H10" s="7" t="n">
+        <v>11</v>
       </c>
       <c r="I10" s="7" t="n">
         <v>7</v>
@@ -993,10 +985,8 @@
           <t>28 Oct 2026 update</t>
         </is>
       </c>
-      <c r="H12" s="7" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
+      <c r="H12" s="7" t="n">
+        <v>33</v>
       </c>
       <c r="I12" s="7" t="n">
         <v>6</v>
@@ -1039,10 +1029,8 @@
           <t>28 Oct 2026 update</t>
         </is>
       </c>
-      <c r="H13" s="7" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
+      <c r="H13" s="7" t="n">
+        <v>40</v>
       </c>
       <c r="I13" s="7" t="n">
         <v>6</v>
@@ -1085,10 +1073,8 @@
           <t>28 Oct 2026 update</t>
         </is>
       </c>
-      <c r="H14" s="7" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
+      <c r="H14" s="7" t="n">
+        <v>27</v>
       </c>
       <c r="I14" s="7" t="n">
         <v>5</v>
@@ -1131,10 +1117,8 @@
           <t>28 Oct 2026 update</t>
         </is>
       </c>
-      <c r="H15" s="7" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
+      <c r="H15" s="7" t="n">
+        <v>32</v>
       </c>
       <c r="I15" s="7" t="n">
         <v>5</v>
@@ -2050,7 +2034,11 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="18" t="n"/>
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>27 kg (incl. packing)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -2397,7 +2385,11 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="18" t="n"/>
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>32 kg (incl. packing)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -5821,7 +5813,7 @@
       </c>
       <c r="B17" s="15" t="inlineStr">
         <is>
-          <t>1-1/2" CPVC</t>
+          <t>1-1/2" (Ø38 mm) CPVC</t>
         </is>
       </c>
     </row>
@@ -5833,7 +5825,7 @@
       </c>
       <c r="B18" s="15" t="inlineStr">
         <is>
-          <t>1-1/2" CPVC</t>
+          <t>1-1/2" (Ø38 mm) CPVC</t>
         </is>
       </c>
     </row>
@@ -6034,7 +6026,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>18 kg</t>
+          <t>18 kg (incl. packing)</t>
         </is>
       </c>
     </row>
@@ -7618,7 +7610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B39"/>
+  <dimension ref="A1:B40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -7801,7 +7793,7 @@
       </c>
       <c r="B17" s="15" t="inlineStr">
         <is>
-          <t>1-1/2" (Ø38 mm)</t>
+          <t>1-1/2" (Ø38 mm) CPVC</t>
         </is>
       </c>
     </row>
@@ -7813,125 +7805,129 @@
       </c>
       <c r="B18" s="15" t="inlineStr">
         <is>
-          <t>1-1/2" (Ø38 mm)</t>
+          <t>1-1/2" (Ø38 mm) CPVC</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>Dimensions (W x D x H)</t>
+          <t>Grease Exit Coupling</t>
         </is>
       </c>
       <c r="B19" s="15" t="inlineStr">
         <is>
-          <t>700 x 400 x 300 mm (2.30 x 1.31 x 0.98 ft)</t>
+          <t>3/8" CPVC</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>Ideal For</t>
+          <t>Dimensions (W x D x H)</t>
         </is>
       </c>
       <c r="B20" s="15" t="inlineStr">
         <is>
-          <t>Restaurants, Cloud Kitchens, Cafes, Hotels, Canteens</t>
+          <t>700 x 400 x 300 mm (2.30 x 1.31 x 0.98 ft)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>Warranty</t>
+          <t>Ideal For</t>
         </is>
       </c>
       <c r="B21" s="15" t="inlineStr">
         <is>
-          <t>12 Months (manufacturing defects)</t>
+          <t>Restaurants, Cloud Kitchens, Cafes, Hotels, Canteens</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="14" t="inlineStr">
         <is>
-          <t>Unboxing Requirement</t>
+          <t>Warranty</t>
         </is>
       </c>
       <c r="B22" s="15" t="inlineStr">
         <is>
-          <t>No special requirements; can be unboxed and inspected by the customer</t>
+          <t>12 Months (manufacturing defects)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="14" t="inlineStr">
         <is>
-          <t>Replacement Policy</t>
+          <t>Unboxing Requirement</t>
         </is>
       </c>
       <c r="B23" s="15" t="inlineStr">
         <is>
-          <t>No replacement</t>
+          <t>No special requirements; can be unboxed and inspected by the customer</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>
-          <t>Return Policy</t>
+          <t>Replacement Policy</t>
         </is>
       </c>
       <c r="B24" s="15" t="inlineStr">
         <is>
-          <t>Non-returnable</t>
+          <t>No replacement</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="14" t="inlineStr">
         <is>
-          <t>Unloading Responsibility</t>
+          <t>Return Policy</t>
         </is>
       </c>
       <c r="B25" s="15" t="inlineStr">
         <is>
-          <t>Customer</t>
+          <t>Non-returnable</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="14" t="inlineStr">
         <is>
+          <t>Unloading Responsibility</t>
+        </is>
+      </c>
+      <c r="B26" s="15" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
+        <is>
           <t>Installation &amp; Technical Support</t>
         </is>
       </c>
-      <c r="B26" s="15" t="inlineStr">
+      <c r="B27" s="15" t="inlineStr">
         <is>
           <t>Not included; simple DIY installation</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="13" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="13" t="inlineStr">
         <is>
           <t>Key Features</t>
         </is>
       </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="9" t="inlineStr">
-        <is>
-          <t>Holds 60 litres with a flow capacity of 850 litres per hour, sized for small to mid-size commercial kitchens</t>
-        </is>
-      </c>
-      <c r="B29" s="6" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>Three-chamber separation: perforated basket catches food scraps, baffle plates hold back floating grease, clean water exits through the drain coupling</t>
+          <t>Holds 60 litres with a flow capacity of 850 litres per hour, sized for small to mid-size commercial kitchens</t>
         </is>
       </c>
       <c r="B30" s="6" t="n"/>
@@ -7939,7 +7935,7 @@
     <row r="31">
       <c r="A31" s="9" t="inlineStr">
         <is>
-          <t>Built in SS304 stainless steel: 1.2 mm (18G) body and lid, 1.0 mm (20G) baffle plates, for corrosion resistance in wet areas</t>
+          <t>Three-chamber separation: perforated basket catches food scraps, baffle plates hold back floating grease, clean water exits through the drain coupling</t>
         </is>
       </c>
       <c r="B31" s="6" t="n"/>
@@ -7947,7 +7943,7 @@
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>Removable SS perforated basket with handle for quick daily cleaning</t>
+          <t>Built in SS304 stainless steel: 1.2 mm (18G) body and lid, 1.0 mm (20G) baffle plates, for corrosion resistance in wet areas</t>
         </is>
       </c>
       <c r="B32" s="6" t="n"/>
@@ -7955,7 +7951,7 @@
     <row r="33">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>Top SS lid with handle for easy access and inspection</t>
+          <t>Removable SS perforated basket with handle for quick daily cleaning</t>
         </is>
       </c>
       <c r="B33" s="6" t="n"/>
@@ -7963,7 +7959,7 @@
     <row r="34">
       <c r="A34" s="9" t="inlineStr">
         <is>
-          <t>1-1/2" (Ø38 mm) inlet and outlet for direct connection to sink waste lines</t>
+          <t>Top SS lid with handle for easy access and inspection</t>
         </is>
       </c>
       <c r="B34" s="6" t="n"/>
@@ -7971,7 +7967,7 @@
     <row r="35">
       <c r="A35" s="9" t="inlineStr">
         <is>
-          <t>700 x 400 x 300 mm (2.30 x 1.31 x 0.98 ft) footprint fits under sinks or at floor level</t>
+          <t>1-1/2" (Ø38 mm) inlet and outlet for direct connection to sink waste lines</t>
         </is>
       </c>
       <c r="B35" s="6" t="n"/>
@@ -7979,33 +7975,45 @@
     <row r="36">
       <c r="A36" s="9" t="inlineStr">
         <is>
+          <t>700 x 400 x 300 mm (2.30 x 1.31 x 0.98 ft) footprint fits under sinks or at floor level</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="9" t="inlineStr">
+        <is>
           <t>Simple DIY installation; no special unboxing requirements</t>
         </is>
       </c>
-      <c r="B36" s="6" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="13" t="inlineStr">
+      <c r="B37" s="6" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="13" t="inlineStr">
         <is>
           <t>Weight</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="18" t="n"/>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>23 kg (incl. packing)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="12">
     <mergeCell ref="A30:B30"/>
-    <mergeCell ref="A38:B38"/>
     <mergeCell ref="A29:B29"/>
     <mergeCell ref="A33:B33"/>
-    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="A37:B37"/>
     <mergeCell ref="A32:B32"/>
     <mergeCell ref="A36:B36"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="A31:B31"/>
+    <mergeCell ref="A39:B39"/>
     <mergeCell ref="A34:B34"/>
     <mergeCell ref="A35:B35"/>
   </mergeCells>
@@ -8019,7 +8027,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B39"/>
+  <dimension ref="A1:B40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -8202,7 +8210,7 @@
       </c>
       <c r="B17" s="15" t="inlineStr">
         <is>
-          <t>1-1/2" (Ø38 mm)</t>
+          <t>1-1/2" (Ø38 mm) CPVC</t>
         </is>
       </c>
     </row>
@@ -8214,125 +8222,129 @@
       </c>
       <c r="B18" s="15" t="inlineStr">
         <is>
-          <t>1-1/2" (Ø38 mm)</t>
+          <t>1-1/2" (Ø38 mm) CPVC</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>Dimensions (W x D x H)</t>
+          <t>Grease Exit Coupling</t>
         </is>
       </c>
       <c r="B19" s="15" t="inlineStr">
         <is>
-          <t>800 x 450 x 350 mm (2.62 x 1.48 x 1.15 ft)</t>
+          <t>3/8" CPVC</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>Ideal For</t>
+          <t>Dimensions (W x D x H)</t>
         </is>
       </c>
       <c r="B20" s="15" t="inlineStr">
         <is>
-          <t>Restaurants, Cloud Kitchens, Cafes, Hotels, Canteens</t>
+          <t>800 x 450 x 350 mm (2.62 x 1.48 x 1.15 ft)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>Warranty</t>
+          <t>Ideal For</t>
         </is>
       </c>
       <c r="B21" s="15" t="inlineStr">
         <is>
-          <t>12 Months (manufacturing defects)</t>
+          <t>Restaurants, Cloud Kitchens, Cafes, Hotels, Canteens</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="14" t="inlineStr">
         <is>
-          <t>Unboxing Requirement</t>
+          <t>Warranty</t>
         </is>
       </c>
       <c r="B22" s="15" t="inlineStr">
         <is>
-          <t>No special requirements; can be unboxed and inspected by the customer</t>
+          <t>12 Months (manufacturing defects)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="14" t="inlineStr">
         <is>
-          <t>Replacement Policy</t>
+          <t>Unboxing Requirement</t>
         </is>
       </c>
       <c r="B23" s="15" t="inlineStr">
         <is>
-          <t>No replacement</t>
+          <t>No special requirements; can be unboxed and inspected by the customer</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>
-          <t>Return Policy</t>
+          <t>Replacement Policy</t>
         </is>
       </c>
       <c r="B24" s="15" t="inlineStr">
         <is>
-          <t>Non-returnable</t>
+          <t>No replacement</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="14" t="inlineStr">
         <is>
-          <t>Unloading Responsibility</t>
+          <t>Return Policy</t>
         </is>
       </c>
       <c r="B25" s="15" t="inlineStr">
         <is>
-          <t>Customer</t>
+          <t>Non-returnable</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="14" t="inlineStr">
         <is>
+          <t>Unloading Responsibility</t>
+        </is>
+      </c>
+      <c r="B26" s="15" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
+        <is>
           <t>Installation &amp; Technical Support</t>
         </is>
       </c>
-      <c r="B26" s="15" t="inlineStr">
+      <c r="B27" s="15" t="inlineStr">
         <is>
           <t>Not included; simple DIY installation</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="13" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="13" t="inlineStr">
         <is>
           <t>Key Features</t>
         </is>
       </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="9" t="inlineStr">
-        <is>
-          <t>Holds 85 litres with a flow capacity of 1150 litres per hour, sized for mid to large commercial kitchens</t>
-        </is>
-      </c>
-      <c r="B29" s="6" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>Three-chamber separation: perforated basket catches food scraps, baffle plates hold back floating grease, clean water exits through the drain coupling</t>
+          <t>Holds 85 litres with a flow capacity of 1150 litres per hour, sized for mid to large commercial kitchens</t>
         </is>
       </c>
       <c r="B30" s="6" t="n"/>
@@ -8340,7 +8352,7 @@
     <row r="31">
       <c r="A31" s="9" t="inlineStr">
         <is>
-          <t>Built in SS304 stainless steel: 1.2 mm (18G) body and lid, 1.0 mm (20G) baffle plates, for corrosion resistance in wet areas</t>
+          <t>Three-chamber separation: perforated basket catches food scraps, baffle plates hold back floating grease, clean water exits through the drain coupling</t>
         </is>
       </c>
       <c r="B31" s="6" t="n"/>
@@ -8348,7 +8360,7 @@
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>Removable SS perforated basket with handle for quick daily cleaning</t>
+          <t>Built in SS304 stainless steel: 1.2 mm (18G) body and lid, 1.0 mm (20G) baffle plates, for corrosion resistance in wet areas</t>
         </is>
       </c>
       <c r="B32" s="6" t="n"/>
@@ -8356,7 +8368,7 @@
     <row r="33">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>Top SS lid with handle for easy access and inspection</t>
+          <t>Removable SS perforated basket with handle for quick daily cleaning</t>
         </is>
       </c>
       <c r="B33" s="6" t="n"/>
@@ -8364,7 +8376,7 @@
     <row r="34">
       <c r="A34" s="9" t="inlineStr">
         <is>
-          <t>1-1/2" (Ø38 mm) inlet and outlet for direct connection to sink waste lines</t>
+          <t>Top SS lid with handle for easy access and inspection</t>
         </is>
       </c>
       <c r="B34" s="6" t="n"/>
@@ -8372,7 +8384,7 @@
     <row r="35">
       <c r="A35" s="9" t="inlineStr">
         <is>
-          <t>800 x 450 x 350 mm (2.62 x 1.48 x 1.15 ft) footprint fits under sinks or at floor level</t>
+          <t>1-1/2" (Ø38 mm) inlet and outlet for direct connection to sink waste lines</t>
         </is>
       </c>
       <c r="B35" s="6" t="n"/>
@@ -8380,33 +8392,45 @@
     <row r="36">
       <c r="A36" s="9" t="inlineStr">
         <is>
+          <t>800 x 450 x 350 mm (2.62 x 1.48 x 1.15 ft) footprint fits under sinks or at floor level</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="9" t="inlineStr">
+        <is>
           <t>Simple DIY installation; no special unboxing requirements</t>
         </is>
       </c>
-      <c r="B36" s="6" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="13" t="inlineStr">
+      <c r="B37" s="6" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="13" t="inlineStr">
         <is>
           <t>Weight</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="18" t="n"/>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>27 kg (incl. packing)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="12">
     <mergeCell ref="A30:B30"/>
-    <mergeCell ref="A38:B38"/>
     <mergeCell ref="A29:B29"/>
     <mergeCell ref="A33:B33"/>
-    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="A37:B37"/>
     <mergeCell ref="A32:B32"/>
     <mergeCell ref="A36:B36"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="A31:B31"/>
+    <mergeCell ref="A39:B39"/>
     <mergeCell ref="A34:B34"/>
     <mergeCell ref="A35:B35"/>
   </mergeCells>
@@ -8742,7 +8766,11 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="18" t="n"/>
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>7 kg (incl. packing)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -9089,7 +9117,11 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="18" t="n"/>
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>11 kg (incl. packing)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -9785,7 +9817,11 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="18" t="n"/>
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>33 kg (incl. packing)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -10132,7 +10168,11 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="18" t="n"/>
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>40 kg (incl. packing)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>

<commit_message>
S.No 6 is the 1150x600 table (4WTU2), not 1050
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KXQyatQdYSKeTsiHbQVdrE
</commit_message>
<xml_diff>
--- a/listing/USP/USP_Listings.xlsx
+++ b/listing/USP/USP_Listings.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 GT84H3H" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 DG11" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 DG21" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 SS_WT_US2_1050" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 4WTU2" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 5TR3" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 5TR4" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 MSR94H" sheetId="10" state="visible" r:id="rId10"/>
@@ -80,7 +80,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -105,11 +105,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -183,7 +178,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -222,7 +217,6 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -916,7 +910,7 @@
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>To confirm</t>
+          <t>4WTU2</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr">
@@ -926,30 +920,26 @@
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>USP Essentials - Stainless Steel Work Table with 2 Under Shelves, 3.44 x 1.97 x 2.79 ft</t>
-        </is>
-      </c>
-      <c r="F11" s="10" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
+          <t>USP Essentials - Stainless Steel Work Table with 2 Under Shelves, 3.77 x 1.97 x 2.79 ft</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="n">
+        <v>21600</v>
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
-          <t>To confirm (1050 mm size not in catalogue)</t>
-        </is>
-      </c>
-      <c r="H11" s="7" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
+          <t>28 Oct 2026 update</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="n">
+        <v>28</v>
       </c>
       <c r="I11" s="7" t="n">
         <v>6</v>
       </c>
       <c r="J11" s="11" t="inlineStr">
         <is>
-          <t>images/06_SS_WT_US2_1050</t>
+          <t>images/06_SS_WT_US2_1150_4WTU2</t>
         </is>
       </c>
     </row>
@@ -9180,7 +9170,7 @@
       </c>
       <c r="B3" s="16" t="inlineStr">
         <is>
-          <t>USP Essentials - Stainless Steel Work Table with 2 Under Shelves, 3.44 x 1.97 x 2.79 ft</t>
+          <t>USP Essentials - Stainless Steel Work Table with 2 Under Shelves, 3.77 x 1.97 x 2.79 ft</t>
         </is>
       </c>
     </row>
@@ -9192,7 +9182,7 @@
       </c>
       <c r="B4" s="15" t="inlineStr">
         <is>
-          <t>To confirm</t>
+          <t>4WTU2</t>
         </is>
       </c>
     </row>
@@ -9202,10 +9192,8 @@
           <t>Price (Rs, excl. GST)</t>
         </is>
       </c>
-      <c r="B5" s="17" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
+      <c r="B5" s="17" t="n">
+        <v>21600</v>
       </c>
     </row>
     <row r="6">
@@ -9216,7 +9204,7 @@
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>To confirm (1050 mm size not in catalogue)</t>
+          <t>28 Oct 2026 update</t>
         </is>
       </c>
     </row>
@@ -9228,7 +9216,7 @@
       </c>
       <c r="B7" s="15" t="inlineStr">
         <is>
-          <t>images/06_SS_WT_US2_1050 (6 images)</t>
+          <t>images/06_SS_WT_US2_1150_4WTU2 (6 images)</t>
         </is>
       </c>
     </row>
@@ -9319,7 +9307,7 @@
       </c>
       <c r="B16" s="15" t="inlineStr">
         <is>
-          <t>1050 x 600 x 850 mm (3.44 x 1.97 x 2.79 ft)</t>
+          <t>1150 x 600 x 850 mm (3.77 x 1.97 x 2.79 ft)</t>
         </is>
       </c>
     </row>
@@ -9417,7 +9405,7 @@
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>1050 x 600 mm worktop at a standard 850 mm working height</t>
+          <t>1150 x 600 mm worktop at a standard 850 mm working height</t>
         </is>
       </c>
       <c r="B26" s="6" t="n"/>
@@ -9470,7 +9458,11 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="18" t="n"/>
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>28 kg (incl. packing)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>

<commit_message>
Add (4WTU2) to S.No 6 product name
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KXQyatQdYSKeTsiHbQVdrE
</commit_message>
<xml_diff>
--- a/listing/USP/USP_Listings.xlsx
+++ b/listing/USP/USP_Listings.xlsx
@@ -611,6 +611,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -920,7 +921,7 @@
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>USP Essentials - Stainless Steel Work Table with 2 Under Shelves, 3.77 x 1.97 x 2.79 ft</t>
+          <t>USP Essentials - Stainless Steel Work Table with 2 Under Shelves, 3.77 x 1.97 x 2.79 ft (4WTU2)</t>
         </is>
       </c>
       <c r="F11" s="10" t="n">
@@ -9170,7 +9171,7 @@
       </c>
       <c r="B3" s="16" t="inlineStr">
         <is>
-          <t>USP Essentials - Stainless Steel Work Table with 2 Under Shelves, 3.77 x 1.97 x 2.79 ft</t>
+          <t>USP Essentials - Stainless Steel Work Table with 2 Under Shelves, 3.77 x 1.97 x 2.79 ft (4WTU2)</t>
         </is>
       </c>
     </row>
@@ -9220,6 +9221,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="13" t="inlineStr">
         <is>
@@ -9395,6 +9397,7 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="13" t="inlineStr">
         <is>
@@ -9450,6 +9453,7 @@
       </c>
       <c r="B31" s="6" t="n"/>
     </row>
+    <row r="32"/>
     <row r="33">
       <c r="A33" s="13" t="inlineStr">
         <is>

</xml_diff>